<commit_message>
Update the eggubator Altium libraries and BOM export
Binary Altium artifacts (SchLib, PcbLib) plus the regenerated Bill of
Materials spreadsheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/eggubator/Project Outputs for eggubator/BOM/Copy of Bill of Materials-eggubator.xlsx
+++ b/hardware/eggubator/Project Outputs for eggubator/BOM/Copy of Bill of Materials-eggubator.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_Workspace\eggAPP\hardware\eggubator\Project Outputs for eggubator\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3093F3CC-55F0-41F2-894A-AE767693C4C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2D76863-6099-4DC5-B908-A3EA476A78CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F89E0A9D-A388-4030-948F-F4B02853452D}"/>
   </bookViews>
@@ -472,7 +472,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -503,6 +503,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -651,7 +657,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -659,9 +665,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -676,9 +679,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -695,9 +695,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -713,7 +710,26 @@
     <xf numFmtId="166" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -729,10 +745,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1074,7 +1086,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74C789DC-4172-4A5A-8B3F-2052EE4D81FD}">
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.33203125" customWidth="1"/>
@@ -1089,16 +1101,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -1123,7 +1135,7 @@
       </c>
       <c r="E3" s="4">
         <f ca="1">TODAY()</f>
-        <v>46249</v>
+        <v>46258</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -1138,835 +1150,838 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" s="7" t="s">
+      <c r="B6" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="I6" s="8" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="25">
+    <row r="7" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="27">
         <f>ROW()-6</f>
         <v>1</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="29" t="s">
+      <c r="E7" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="12"/>
-      <c r="G7" s="27">
+      <c r="F7" s="30"/>
+      <c r="G7" s="31">
         <v>2</v>
       </c>
-      <c r="H7" s="13">
-        <v>0</v>
-      </c>
-      <c r="I7" s="14">
+      <c r="H7" s="32">
+        <v>0</v>
+      </c>
+      <c r="I7" s="33">
         <f>G7*H7</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="26">
+    <row r="8" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="27">
         <f t="shared" ref="A8:A33" si="0">ROW()-6</f>
         <v>2</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="28">
+      <c r="F8" s="30"/>
+      <c r="G8" s="31">
         <v>2</v>
       </c>
-      <c r="H8" s="23">
-        <v>0</v>
-      </c>
-      <c r="I8" s="24">
+      <c r="H8" s="32">
+        <v>0</v>
+      </c>
+      <c r="I8" s="33">
         <f t="shared" ref="I8:I33" si="1">G8*H8</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="25">
+    <row r="9" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="27">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="12"/>
-      <c r="G9" s="27">
+      <c r="F9" s="30"/>
+      <c r="G9" s="31">
         <v>3</v>
       </c>
-      <c r="H9" s="13">
-        <v>0</v>
-      </c>
-      <c r="I9" s="14">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="26">
+      <c r="H9" s="32">
+        <v>0</v>
+      </c>
+      <c r="I9" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="27">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="D10" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="22"/>
-      <c r="G10" s="28">
+      <c r="F10" s="30"/>
+      <c r="G10" s="31">
         <v>6</v>
       </c>
-      <c r="H10" s="23">
-        <v>0</v>
-      </c>
-      <c r="I10" s="24">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="25">
+      <c r="H10" s="32">
+        <v>0</v>
+      </c>
+      <c r="I10" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="27">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="12"/>
-      <c r="G11" s="27">
+      <c r="F11" s="30"/>
+      <c r="G11" s="31">
         <v>1</v>
       </c>
-      <c r="H11" s="13">
-        <v>0</v>
-      </c>
-      <c r="I11" s="14">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="26">
+      <c r="H11" s="32">
+        <v>0</v>
+      </c>
+      <c r="I11" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="27">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="22" t="s">
+      <c r="E12" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="F12" s="22"/>
-      <c r="G12" s="28">
+      <c r="F12" s="30"/>
+      <c r="G12" s="31">
         <v>1</v>
       </c>
-      <c r="H12" s="23">
-        <v>0</v>
-      </c>
-      <c r="I12" s="24">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="25">
+      <c r="H12" s="32">
+        <v>0</v>
+      </c>
+      <c r="I12" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="27">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="F13" s="12"/>
-      <c r="G13" s="27">
+      <c r="F13" s="30"/>
+      <c r="G13" s="31">
         <v>1</v>
       </c>
-      <c r="H13" s="13">
-        <v>0</v>
-      </c>
-      <c r="I13" s="14">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="26">
+      <c r="H13" s="32">
+        <v>0</v>
+      </c>
+      <c r="I13" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="27">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="D14" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="E14" s="22" t="s">
+      <c r="E14" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="F14" s="22"/>
-      <c r="G14" s="28">
+      <c r="F14" s="30"/>
+      <c r="G14" s="31">
         <v>1</v>
       </c>
-      <c r="H14" s="23">
-        <v>0</v>
-      </c>
-      <c r="I14" s="24">
+      <c r="H14" s="32">
+        <v>0</v>
+      </c>
+      <c r="I14" s="33">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="25">
+      <c r="A15" s="22">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="10">
         <v>691137710003</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="10">
         <v>691137710003</v>
       </c>
-      <c r="F15" s="12"/>
-      <c r="G15" s="27">
+      <c r="F15" s="10"/>
+      <c r="G15" s="24">
         <v>8</v>
       </c>
-      <c r="H15" s="13">
-        <v>0</v>
-      </c>
-      <c r="I15" s="14">
+      <c r="H15" s="11">
+        <v>0</v>
+      </c>
+      <c r="I15" s="12">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="26">
+      <c r="A16" s="23">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="19">
         <v>2828372</v>
       </c>
-      <c r="E16" s="22" t="s">
+      <c r="E16" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="F16" s="22"/>
-      <c r="G16" s="28">
+      <c r="F16" s="19"/>
+      <c r="G16" s="25">
         <v>1</v>
       </c>
-      <c r="H16" s="23">
-        <v>0</v>
-      </c>
-      <c r="I16" s="24">
+      <c r="H16" s="20">
+        <v>0</v>
+      </c>
+      <c r="I16" s="21">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="25">
+      <c r="A17" s="22">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="12">
+      <c r="D17" s="10">
         <v>2828375</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="F17" s="12"/>
-      <c r="G17" s="27">
+      <c r="F17" s="10"/>
+      <c r="G17" s="24">
         <v>1</v>
       </c>
-      <c r="H17" s="13">
-        <v>0</v>
-      </c>
-      <c r="I17" s="14">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="26">
+      <c r="H17" s="11">
+        <v>0</v>
+      </c>
+      <c r="I17" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="27">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="E18" s="22" t="s">
+      <c r="E18" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="F18" s="22"/>
-      <c r="G18" s="28">
+      <c r="F18" s="30"/>
+      <c r="G18" s="31">
         <v>6</v>
       </c>
-      <c r="H18" s="23">
-        <v>0</v>
-      </c>
-      <c r="I18" s="24">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="25">
+      <c r="H18" s="32">
+        <v>0</v>
+      </c>
+      <c r="I18" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="27">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="F19" s="12"/>
-      <c r="G19" s="27">
+      <c r="F19" s="30"/>
+      <c r="G19" s="31">
         <v>1</v>
       </c>
-      <c r="H19" s="13">
-        <v>0</v>
-      </c>
-      <c r="I19" s="14">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="26">
+      <c r="H19" s="32">
+        <v>0</v>
+      </c>
+      <c r="I19" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="27">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="22" t="s">
+      <c r="D20" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="E20" s="22" t="s">
+      <c r="E20" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="F20" s="22"/>
-      <c r="G20" s="28">
+      <c r="F20" s="30"/>
+      <c r="G20" s="31">
         <v>6</v>
       </c>
-      <c r="H20" s="23">
-        <v>0</v>
-      </c>
-      <c r="I20" s="24">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="25">
+      <c r="H20" s="32">
+        <v>0</v>
+      </c>
+      <c r="I20" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="27">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="F21" s="12"/>
-      <c r="G21" s="27">
+      <c r="F21" s="30"/>
+      <c r="G21" s="31">
         <v>2</v>
       </c>
-      <c r="H21" s="13">
-        <v>0</v>
-      </c>
-      <c r="I21" s="14">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="26">
+      <c r="H21" s="32">
+        <v>0</v>
+      </c>
+      <c r="I21" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="27">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="B22" s="20" t="s">
+      <c r="B22" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="C22" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="D22" s="22" t="s">
+      <c r="D22" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="E22" s="22" t="s">
+      <c r="E22" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="F22" s="22"/>
-      <c r="G22" s="28">
+      <c r="F22" s="30"/>
+      <c r="G22" s="31">
         <v>1</v>
       </c>
-      <c r="H22" s="23">
-        <v>0</v>
-      </c>
-      <c r="I22" s="24">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="25">
+      <c r="H22" s="32">
+        <v>0</v>
+      </c>
+      <c r="I22" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="27">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="D23" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="E23" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="F23" s="12"/>
-      <c r="G23" s="27">
+      <c r="F23" s="30"/>
+      <c r="G23" s="31">
         <v>2</v>
       </c>
-      <c r="H23" s="13">
-        <v>0</v>
-      </c>
-      <c r="I23" s="14">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="26">
+      <c r="H23" s="32">
+        <v>0</v>
+      </c>
+      <c r="I23" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="27">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="B24" s="20" t="s">
+      <c r="B24" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="C24" s="20" t="s">
+      <c r="C24" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="D24" s="22" t="s">
+      <c r="D24" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="E24" s="22" t="s">
+      <c r="E24" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="F24" s="22"/>
-      <c r="G24" s="28">
+      <c r="F24" s="30"/>
+      <c r="G24" s="31">
         <v>1</v>
       </c>
-      <c r="H24" s="23">
-        <v>0</v>
-      </c>
-      <c r="I24" s="24">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="25">
+      <c r="H24" s="32">
+        <v>0</v>
+      </c>
+      <c r="I24" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="27">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="D25" s="12" t="s">
+      <c r="D25" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E25" s="12" t="s">
+      <c r="E25" s="30" t="s">
         <v>68</v>
       </c>
-      <c r="F25" s="12"/>
-      <c r="G25" s="27">
+      <c r="F25" s="30"/>
+      <c r="G25" s="31">
         <v>1</v>
       </c>
-      <c r="H25" s="13">
-        <v>0</v>
-      </c>
-      <c r="I25" s="14">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="26">
+      <c r="H25" s="32">
+        <v>0</v>
+      </c>
+      <c r="I25" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="27">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="C26" s="20" t="s">
+      <c r="C26" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="D26" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="E26" s="22" t="s">
+      <c r="E26" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="F26" s="22"/>
-      <c r="G26" s="28">
+      <c r="F26" s="30"/>
+      <c r="G26" s="31">
         <v>1</v>
       </c>
-      <c r="H26" s="23">
-        <v>0</v>
-      </c>
-      <c r="I26" s="24">
+      <c r="H26" s="32">
+        <v>0</v>
+      </c>
+      <c r="I26" s="33">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="25">
+      <c r="A27" s="22">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D27" s="12" t="s">
+      <c r="D27" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="E27" s="12" t="s">
+      <c r="E27" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="F27" s="12"/>
-      <c r="G27" s="27">
+      <c r="F27" s="10"/>
+      <c r="G27" s="24">
         <v>6</v>
       </c>
-      <c r="H27" s="13">
-        <v>0</v>
-      </c>
-      <c r="I27" s="14">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="26">
+      <c r="H27" s="11">
+        <v>0</v>
+      </c>
+      <c r="I27" s="12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="27">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="B28" s="20" t="s">
+      <c r="B28" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="C28" s="20" t="s">
+      <c r="C28" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="D28" s="22" t="s">
+      <c r="D28" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="E28" s="22" t="s">
+      <c r="E28" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="F28" s="22"/>
-      <c r="G28" s="28">
+      <c r="F28" s="30"/>
+      <c r="G28" s="31">
         <v>8</v>
       </c>
-      <c r="H28" s="23">
-        <v>0</v>
-      </c>
-      <c r="I28" s="24">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="25">
+      <c r="H28" s="32">
+        <v>0</v>
+      </c>
+      <c r="I28" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="27">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="28" t="s">
         <v>81</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="D29" s="12" t="s">
+      <c r="D29" s="30" t="s">
         <v>83</v>
       </c>
-      <c r="E29" s="12" t="s">
+      <c r="E29" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="F29" s="12"/>
-      <c r="G29" s="27">
+      <c r="F29" s="30"/>
+      <c r="G29" s="31">
         <v>6</v>
       </c>
-      <c r="H29" s="13">
-        <v>0</v>
-      </c>
-      <c r="I29" s="14">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="26">
+      <c r="H29" s="32">
+        <v>0</v>
+      </c>
+      <c r="I29" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="27">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="B30" s="20" t="s">
+      <c r="B30" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="C30" s="20" t="s">
+      <c r="C30" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="D30" s="22" t="s">
+      <c r="D30" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="E30" s="22" t="s">
+      <c r="E30" s="30" t="s">
         <v>88</v>
       </c>
-      <c r="F30" s="22"/>
-      <c r="G30" s="28">
+      <c r="F30" s="30"/>
+      <c r="G30" s="31">
         <v>6</v>
       </c>
-      <c r="H30" s="23">
-        <v>0</v>
-      </c>
-      <c r="I30" s="24">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="25">
+      <c r="H30" s="32">
+        <v>0</v>
+      </c>
+      <c r="I30" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="27">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="28" t="s">
         <v>89</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="D31" s="12" t="s">
+      <c r="D31" s="30" t="s">
         <v>83</v>
       </c>
-      <c r="E31" s="12" t="s">
+      <c r="E31" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="F31" s="12"/>
-      <c r="G31" s="27">
+      <c r="F31" s="30"/>
+      <c r="G31" s="31">
         <v>1</v>
       </c>
-      <c r="H31" s="13">
-        <v>0</v>
-      </c>
-      <c r="I31" s="14">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="26">
+      <c r="H31" s="32">
+        <v>0</v>
+      </c>
+      <c r="I31" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="27">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="B32" s="20" t="s">
+      <c r="B32" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="C32" s="20" t="s">
+      <c r="C32" s="28" t="s">
         <v>93</v>
       </c>
-      <c r="D32" s="22" t="s">
+      <c r="D32" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="E32" s="22" t="s">
+      <c r="E32" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="F32" s="22"/>
-      <c r="G32" s="28">
+      <c r="F32" s="30"/>
+      <c r="G32" s="31">
         <v>3</v>
       </c>
-      <c r="H32" s="23">
-        <v>0</v>
-      </c>
-      <c r="I32" s="24">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="25">
+      <c r="H32" s="32">
+        <v>0</v>
+      </c>
+      <c r="I32" s="33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="27">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="D33" s="12" t="s">
+      <c r="D33" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="E33" s="12" t="s">
+      <c r="E33" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="F33" s="12"/>
-      <c r="G33" s="27">
+      <c r="F33" s="30"/>
+      <c r="G33" s="31">
         <v>2</v>
       </c>
-      <c r="H33" s="13">
-        <v>0</v>
-      </c>
-      <c r="I33" s="14">
+      <c r="H33" s="32">
+        <v>0</v>
+      </c>
+      <c r="I33" s="33">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="15"/>
-      <c r="B34" s="16"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="17" t="s">
+      <c r="A34" s="13"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="H34" s="18">
+      <c r="H34" s="16">
         <f>SUM(G7:G33)</f>
         <v>80</v>
       </c>
-      <c r="I34" s="19">
+      <c r="I34" s="17">
         <f>SUM(I7:I33)</f>
         <v>0</v>
       </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C37" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>